<commit_message>
Fujairah 3-site split + N/A filter fix
</commit_message>
<xml_diff>
--- a/ITR_Status_Report.xlsx
+++ b/ITR_Status_Report.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITR Status" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ITR Status'!$A$1:$G$434</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ITR Status'!$A$1:$G$435</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G434"/>
+  <dimension ref="A1:G435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -771,7 +771,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -904,7 +904,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -933,7 +933,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -8218,7 +8218,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>CODE-2</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="E244" t="inlineStr"/>
@@ -12785,12 +12785,12 @@
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Track Laying</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -12814,12 +12814,12 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Ballast MATS</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
@@ -12843,12 +12843,12 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Ballast Mats(future Line)</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
@@ -12872,12 +12872,12 @@
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Turnout Installation</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
@@ -12901,12 +12901,12 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>MFBW</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
@@ -12930,12 +12930,12 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Turnout 1st Tamping</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
@@ -12959,12 +12959,12 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Turnout 2nd Tamping</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -12988,12 +12988,12 @@
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Turnout 3rd Tamping</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
@@ -13017,12 +13017,12 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Turnout Final Tamping</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
@@ -13046,12 +13046,12 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>ATW</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
@@ -13075,12 +13075,12 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Turnout De-stressing</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -13104,12 +13104,12 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>De-streesing Of Rail</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -13133,12 +13133,12 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>1sttamping</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -13162,12 +13162,12 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>2nd Tamping</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -13191,12 +13191,12 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>3rd Tamping</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -13220,12 +13220,12 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Final Tamping</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -13249,12 +13249,12 @@
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Ballast Profilling</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -13278,12 +13278,12 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Control Point</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -13307,12 +13307,12 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Fujairah Clearance And Fouling Marker</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -13336,12 +13336,12 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Structural Gauge</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -13365,12 +13365,12 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Track Maker</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -13394,12 +13394,12 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Station</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>Fujirah Station</t>
+          <t>Buffer Stop</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
@@ -13423,12 +13423,12 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Loop</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>Fujirah-New</t>
+          <t>Existing Track Removal</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
@@ -13438,7 +13438,7 @@
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>未匹配到对应code</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="E416" t="inlineStr">
@@ -13448,24 +13448,24 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>FPJ 01A</t>
+          <t>HJR19A</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
         <is>
-          <t>CH 55+002</t>
+          <t>CH 48+887</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Loop</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Fujirah-New</t>
+          <t>Existing Track Removal</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -13475,7 +13475,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>未匹配到对应code</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="E417" t="inlineStr">
@@ -13485,24 +13485,24 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>HJR19A</t>
+          <t>HJR19B</t>
         </is>
       </c>
       <c r="G417" t="inlineStr">
         <is>
-          <t>CH 48+887</t>
+          <t>CH 50+942</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Loop</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>Fujirah-New</t>
+          <t>Track Laying</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -13512,34 +13512,34 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>未匹配到对应code</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>Existing Track removal</t>
+          <t>Track laying</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>HJR19B</t>
+          <t>HJR</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
         <is>
-          <t>CH 50+942</t>
+          <t>CH 48+927</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Loop</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>Fujirah-New</t>
+          <t>Ballast Mat</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -13549,34 +13549,34 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>未匹配到对应code</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>Track laying</t>
+          <t>ballast mat</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t>FJP</t>
+          <t>HJR</t>
         </is>
       </c>
       <c r="G419" t="inlineStr">
         <is>
-          <t>CH 55+041</t>
+          <t>CH 50+200</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Port</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Fujirah-New</t>
+          <t>Existing Track Removal</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -13586,34 +13586,34 @@
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>未匹配到对应code</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>Track laying</t>
+          <t>Existing Track removal</t>
         </is>
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>FJP</t>
+          <t>FPJ 01A</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
         <is>
-          <t>CH 55+543</t>
+          <t>CH 55+002</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Port</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>Fujirah-New</t>
+          <t>Track Laying</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>未匹配到对应code</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="E421" t="inlineStr">
@@ -13638,19 +13638,19 @@
       </c>
       <c r="G421" t="inlineStr">
         <is>
-          <t>CH 55+041</t>
+          <t>CH 55+543</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Port</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Fujirah-New</t>
+          <t>Bottom Ballast</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -13660,34 +13660,34 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>未匹配到对应code</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>Track laying</t>
+          <t>bottom ballast</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t>HJR</t>
+          <t>FJP</t>
         </is>
       </c>
       <c r="G422" t="inlineStr">
         <is>
-          <t>CH 48+927</t>
+          <t>CH 55+543</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>Fujairah</t>
+          <t>Fujairah Port</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>Fujirah-New</t>
+          <t>Bottom Ballast</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -13697,7 +13697,7 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>未匹配到对应code</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="E423" t="inlineStr">
@@ -13712,36 +13712,44 @@
       </c>
       <c r="G423" t="inlineStr">
         <is>
-          <t>CH 55+543</t>
+          <t>CH 55+043</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>LIWA</t>
+          <t>Fujairah Port</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Liwa</t>
+          <t>Track Laying</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>P2414-GMC-GQC-IR-00243</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>CODE-2</t>
-        </is>
-      </c>
-      <c r="E424" t="inlineStr"/>
-      <c r="F424" t="inlineStr"/>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Track laying</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>FJP</t>
+        </is>
+      </c>
       <c r="G424" t="inlineStr">
         <is>
-          <t>CH 01+100</t>
+          <t>CH 55+043</t>
         </is>
       </c>
     </row>
@@ -13753,12 +13761,12 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>Liwa</t>
+          <t>Track Laying</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>P2414-GMC-GQC-IR-00251</t>
+          <t>P2414-GMC-GQC-IR-00243</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
@@ -13770,7 +13778,7 @@
       <c r="F425" t="inlineStr"/>
       <c r="G425" t="inlineStr">
         <is>
-          <t>CH 00+250</t>
+          <t>CH 01+100</t>
         </is>
       </c>
     </row>
@@ -13782,24 +13790,24 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Liwa</t>
+          <t>Track Laying</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>P2414-GMC-GQC-IR-00253</t>
+          <t>P2414-GMC-GQC-IR-00251</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E426" t="inlineStr"/>
       <c r="F426" t="inlineStr"/>
       <c r="G426" t="inlineStr">
         <is>
-          <t>CH 00+000</t>
+          <t>CH 00+250</t>
         </is>
       </c>
     </row>
@@ -13811,24 +13819,24 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>Liwa</t>
+          <t>Track Laying</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>P2414-GMC-GQC-IR-00244</t>
+          <t>P2414-GMC-GQC-IR-00253</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>CODE-2</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="E427" t="inlineStr"/>
       <c r="F427" t="inlineStr"/>
       <c r="G427" t="inlineStr">
         <is>
-          <t>CH 01+100</t>
+          <t>CH 00+000</t>
         </is>
       </c>
     </row>
@@ -13840,24 +13848,24 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>Liwa</t>
+          <t>Bottom Ballast</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>P2414-GMC-GQC-IR-00250</t>
+          <t>P2414-GMC-GQC-IR-00244</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>CODE-3</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E428" t="inlineStr"/>
       <c r="F428" t="inlineStr"/>
       <c r="G428" t="inlineStr">
         <is>
-          <t>CH 00+250</t>
+          <t>CH 01+100</t>
         </is>
       </c>
     </row>
@@ -13869,24 +13877,24 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>Liwa</t>
+          <t>Bottom Ballast</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>P2414-GMC-GQC-IR-00245</t>
+          <t>P2414-GMC-GQC-IR-00250</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>CODE-2</t>
+          <t>CODE-3</t>
         </is>
       </c>
       <c r="E429" t="inlineStr"/>
       <c r="F429" t="inlineStr"/>
       <c r="G429" t="inlineStr">
         <is>
-          <t>CH 02+785</t>
+          <t>CH 00+250</t>
         </is>
       </c>
     </row>
@@ -13898,24 +13906,24 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>Liwa</t>
+          <t>Existing Track Ramoval</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>P2414-GMC-GQC-IR-00254</t>
+          <t>P2414-GMC-GQC-IR-00245</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E430" t="inlineStr"/>
       <c r="F430" t="inlineStr"/>
       <c r="G430" t="inlineStr">
         <is>
-          <t>CH 02+266</t>
+          <t>CH 02+785</t>
         </is>
       </c>
     </row>
@@ -13927,51 +13935,51 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>Liwa</t>
+          <t>Existing Track Ramoval</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>P2414-GMC-GQC-IR-00247</t>
+          <t>P2414-GMC-GQC-IR-00254</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>CODE-3</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="E431" t="inlineStr"/>
       <c r="F431" t="inlineStr"/>
-      <c r="G431" t="inlineStr"/>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>CH 02+266</t>
+        </is>
+      </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>PL-28</t>
+          <t>LIWA</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>PL-28</t>
+          <t>Turnout Installation</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>P2216-DMB-GQC-IR-00360</t>
+          <t>P2414-GMC-GQC-IR-00247</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>CODE-2</t>
+          <t>CODE-3</t>
         </is>
       </c>
       <c r="E432" t="inlineStr"/>
       <c r="F432" t="inlineStr"/>
-      <c r="G432" t="inlineStr">
-        <is>
-          <t>CH 28+414</t>
-        </is>
-      </c>
+      <c r="G432" t="inlineStr"/>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -13981,24 +13989,24 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>PL-28</t>
+          <t>Track Laying</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>P2216-DMB-GQC-IR-00328</t>
+          <t>P2216-DMB-GQC-IR-00360</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>CODE-2</t>
         </is>
       </c>
       <c r="E433" t="inlineStr"/>
       <c r="F433" t="inlineStr"/>
       <c r="G433" t="inlineStr">
         <is>
-          <t>CH 28+425</t>
+          <t>CH 28+414</t>
         </is>
       </c>
     </row>
@@ -14010,29 +14018,58 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>PL-28</t>
+          <t>Bottom Ballast</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>P2216-DMB-GQC-IR-00359</t>
+          <t>P2216-DMB-GQC-IR-00328</t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="E434" t="inlineStr"/>
       <c r="F434" t="inlineStr"/>
       <c r="G434" t="inlineStr">
         <is>
+          <t>CH 28+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>PL-28</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Bottom Ballast</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>P2216-DMB-GQC-IR-00359</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr"/>
+      <c r="F435" t="inlineStr"/>
+      <c r="G435" t="inlineStr">
+        <is>
           <t>CH 29+500</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G434"/>
+  <autoFilter ref="A1:G435"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>